<commit_message>
Atualizar planilhas CVM [2026-03-11]
</commit_message>
<xml_diff>
--- a/patrimonio_liquido_cvm_08915927.xlsx
+++ b/patrimonio_liquido_cvm_08915927.xlsx
@@ -667,7 +667,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C6"/>
+  <dimension ref="A1:G6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -686,6 +686,26 @@
           <t>Share</t>
         </is>
       </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>A/P</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Risco</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>Negocio/Banca</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -699,6 +719,10 @@
       <c r="C2" t="n">
         <v>0.7554155888736424</v>
       </c>
+      <c r="D2" t="inlineStr"/>
+      <c r="E2" t="inlineStr"/>
+      <c r="F2" t="inlineStr"/>
+      <c r="G2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -712,6 +736,26 @@
       <c r="C3" t="n">
         <v>0.2441792307438946</v>
       </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>A10</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>JP2</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>02</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -725,6 +769,26 @@
       <c r="C4" t="n">
         <v>0.0002872703390889405</v>
       </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>A10</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>998</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>02</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>02</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -738,6 +802,26 @@
       <c r="C5" t="n">
         <v>0.0001152250261697982</v>
       </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>P90</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>998</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>02</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>02</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -750,6 +834,26 @@
       </c>
       <c r="C6" t="n">
         <v>2.685017204352634e-06</v>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>A90</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>998</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>02</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>02</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Atualizar planilhas CVM [2026-04-08]
</commit_message>
<xml_diff>
--- a/patrimonio_liquido_cvm_08915927.xlsx
+++ b/patrimonio_liquido_cvm_08915927.xlsx
@@ -462,7 +462,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>02/2026</t>
+          <t>03/2026</t>
         </is>
       </c>
     </row>
@@ -474,7 +474,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>R$ 27.376.309.196,54</t>
+          <t>R$ 28.512.890.821,01</t>
         </is>
       </c>
     </row>
@@ -486,7 +486,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>05/03/2026 14:25:18</t>
+          <t>08/04/2026 11:35:16</t>
         </is>
       </c>
     </row>
@@ -523,27 +523,27 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>7866235.31</v>
+        <v>586655.42</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Operações Compromissadas Cod. SELIC: 100000 Venc.: 01/01/2029</t>
+          <t>Operações Compromissadas Cod. SELIC: 100000 Venc.: 01/01/2032</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>4492619539.5</v>
+        <v>5135244601.77</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Operações Compromissadas Cod. SELIC: 950199 Venc.: 01/01/2029</t>
+          <t>Operações Compromissadas Cod. SELIC: 950199 Venc.: 01/01/2027</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>2193665208.65</v>
+        <v>2617849830.11</v>
       </c>
     </row>
     <row r="5">
@@ -553,7 +553,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>8195811298.63</v>
+        <v>7972131716.9</v>
       </c>
     </row>
     <row r="6">
@@ -563,7 +563,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>3398933538.09</v>
+        <v>3144363940.14</v>
       </c>
     </row>
     <row r="7">
@@ -573,7 +573,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>3067815717.22</v>
+        <v>3001636423.26</v>
       </c>
     </row>
     <row r="8">
@@ -583,7 +583,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>2227581157.19</v>
+        <v>2320839118.33</v>
       </c>
     </row>
     <row r="9">
@@ -593,27 +593,27 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>1579098012.86</v>
+        <v>1599675324.27</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Títulos Públicos Cod. SELIC: 210100 Venc.: 01/03/2030</t>
+          <t>Títulos Públicos Cod. SELIC: 210100 Venc.: 01/09/2029</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>1025819021.27</v>
+        <v>1248030038.81</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Títulos Públicos Cod. SELIC: 210100 Venc.: 01/09/2029</t>
+          <t>Títulos Públicos Cod. SELIC: 210100 Venc.: 01/03/2030</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>679121922.52</v>
+        <v>1094278640.23</v>
       </c>
     </row>
     <row r="12">
@@ -623,17 +623,17 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>463364785.09</v>
+        <v>381680506.45</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Títulos Públicos Cod. SELIC: 210100 Venc.: 01/03/2026</t>
+          <t>Títulos Públicos Cod. SELIC: 210100 Venc.: 01/09/2030</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>47767196.42</v>
+        <v>186421.04</v>
       </c>
     </row>
     <row r="14">
@@ -643,7 +643,7 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>3155171.44</v>
+        <v>3612395.72</v>
       </c>
     </row>
     <row r="15">
@@ -653,7 +653,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>73523</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -714,10 +714,10 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>20685312649.29</v>
+        <v>20762822129.43</v>
       </c>
       <c r="C2" t="n">
-        <v>0.7554155888736424</v>
+        <v>0.728006239931451</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
@@ -747,10 +747,10 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>6686284748.15</v>
+        <v>7753094431.880001</v>
       </c>
       <c r="C3" t="n">
-        <v>0.2441792307438946</v>
+        <v>0.2718465288582319</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
@@ -776,18 +776,18 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Disponibilidades</t>
+          <t>Valores a pagar</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>7866235.31</v>
+        <v>3612395.72</v>
       </c>
       <c r="C4" t="n">
-        <v>0.0002872703390889405</v>
+        <v>0.0001266613280635884</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>A10</t>
+          <t>P90</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -809,18 +809,18 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Valores a pagar</t>
+          <t>Disponibilidades</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>3155171.44</v>
+        <v>586655.42</v>
       </c>
       <c r="C5" t="n">
-        <v>0.0001152250261697982</v>
+        <v>2.05698822533491e-05</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>P90</t>
+          <t>A10</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -846,10 +846,10 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>73523</v>
+        <v>0</v>
       </c>
       <c r="C6" t="n">
-        <v>2.685017204352634e-06</v>
+        <v>0</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>

</xml_diff>